<commit_message>
fix #190: rellenar datos uso, user, compania , etc
</commit_message>
<xml_diff>
--- a/RamoProducto.xlsx
+++ b/RamoProducto.xlsx
@@ -5,15 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC1\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC1\OneDrive\Documentos\GitHub\SIS-ARIAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D4F700-B880-4B53-B4D9-C4D278BB0390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FC4832-1BCC-4E16-BDA0-A750EEBC555E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="RamoProducto" sheetId="1" r:id="rId1"/>
+    <sheet name="compania" sheetId="2" r:id="rId2"/>
+    <sheet name="ejecutivo" sheetId="3" r:id="rId3"/>
+    <sheet name="Endosatarios" sheetId="4" r:id="rId4"/>
+    <sheet name="Clases Veh" sheetId="5" r:id="rId5"/>
+    <sheet name="Marca" sheetId="6" r:id="rId6"/>
+    <sheet name="Modelo" sheetId="11" r:id="rId7"/>
+    <sheet name="SubAgent" sheetId="7" r:id="rId8"/>
+    <sheet name="Usuario" sheetId="8" r:id="rId9"/>
+    <sheet name="Uso" sheetId="9" r:id="rId10"/>
+    <sheet name="Ajustadores" sheetId="10" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -70,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="715">
   <si>
     <t>Ramo</t>
   </si>
@@ -1012,6 +1022,1209 @@
   </si>
   <si>
     <t>MULT NEGOC</t>
+  </si>
+  <si>
+    <t>Nombre Corto   </t>
+  </si>
+  <si>
+    <t>Ruc   </t>
+  </si>
+  <si>
+    <t>Tel1   </t>
+  </si>
+  <si>
+    <t>Central de Emergencia   </t>
+  </si>
+  <si>
+    <t>Logo</t>
+  </si>
+  <si>
+    <t>Rimac</t>
+  </si>
+  <si>
+    <t> 993175447</t>
+  </si>
+  <si>
+    <t>Pacífico</t>
+  </si>
+  <si>
+    <t>PACIFICO</t>
+  </si>
+  <si>
+    <t>La Positiva</t>
+  </si>
+  <si>
+    <t>POSITIVA</t>
+  </si>
+  <si>
+    <t>HDI</t>
+  </si>
+  <si>
+    <t> 993175448</t>
+  </si>
+  <si>
+    <t>Mapfre</t>
+  </si>
+  <si>
+    <t>MAPFRE</t>
+  </si>
+  <si>
+    <t>SANITAS PERÚ SA - EPS</t>
+  </si>
+  <si>
+    <t>SANITAS</t>
+  </si>
+  <si>
+    <t>CRECER SEGUROS S.A. COMPAÑÍA DE SEGUROS</t>
+  </si>
+  <si>
+    <t>CRECER</t>
+  </si>
+  <si>
+    <t>LA POSITIVA VIDA SEGUROS Y REASEGUROS</t>
+  </si>
+  <si>
+    <t>LPV</t>
+  </si>
+  <si>
+    <t>LA POSITIVA S.A. ENTIDAD PRESTADORA DE SALUD</t>
+  </si>
+  <si>
+    <t>LPEPS</t>
+  </si>
+  <si>
+    <t>PROTECTA SA COMPAÑÍA DE SEGUROS</t>
+  </si>
+  <si>
+    <t>PROTECTA</t>
+  </si>
+  <si>
+    <t>AVLA</t>
+  </si>
+  <si>
+    <t>QUALITAS COMPAÑIA DE SEGUROS</t>
+  </si>
+  <si>
+    <t>QUALITAS</t>
+  </si>
+  <si>
+    <t> 01 2303030</t>
+  </si>
+  <si>
+    <t>OHIO NATIONAL SEGUROS DE VIDA Y REASEGUROS S.A</t>
+  </si>
+  <si>
+    <t>OHIO</t>
+  </si>
+  <si>
+    <t> 01204-2330</t>
+  </si>
+  <si>
+    <t>GRANDIA S.A. ENTIDAD PRESTADORA DE SALUD</t>
+  </si>
+  <si>
+    <t>GRANDIAEPS</t>
+  </si>
+  <si>
+    <t>ANDION RUIZ, MONICA</t>
+  </si>
+  <si>
+    <t>ARM</t>
+  </si>
+  <si>
+    <t>ANTONIO MARTÍNEZ, ANDRES</t>
+  </si>
+  <si>
+    <t>AMA</t>
+  </si>
+  <si>
+    <t>ARIAS MURGADO CESAR AUGUSTO</t>
+  </si>
+  <si>
+    <t>CESAR ARIASM</t>
+  </si>
+  <si>
+    <t>ARIAS Y ARIAS</t>
+  </si>
+  <si>
+    <t>ARROYO RAMOS pamela</t>
+  </si>
+  <si>
+    <t>INTERCONEXION</t>
+  </si>
+  <si>
+    <t>CALDERON LOZADA, WILLIAMS MERCEDES</t>
+  </si>
+  <si>
+    <t>CLWM</t>
+  </si>
+  <si>
+    <t>CAPILLO SALAVERRY GABY GLEDIS</t>
+  </si>
+  <si>
+    <t>CASGGLEDIS</t>
+  </si>
+  <si>
+    <t>CASTILLO SANTA MARÍA ESTHER</t>
+  </si>
+  <si>
+    <t>CASTILLOMARIA</t>
+  </si>
+  <si>
+    <t>DIAZ URIBE, JOSE FERNANDO</t>
+  </si>
+  <si>
+    <t>DUJF</t>
+  </si>
+  <si>
+    <t>FLORES HUANUIRI, BETTY MILENE</t>
+  </si>
+  <si>
+    <t>FHBM</t>
+  </si>
+  <si>
+    <t>GABRIELA RUIZ</t>
+  </si>
+  <si>
+    <t>GABRIELA</t>
+  </si>
+  <si>
+    <t>GUERRA PEREZ, PEDRO ALFONSO</t>
+  </si>
+  <si>
+    <t>GPPA</t>
+  </si>
+  <si>
+    <t>JOSE</t>
+  </si>
+  <si>
+    <t>Soat</t>
+  </si>
+  <si>
+    <t>KEVIN MURRIETA</t>
+  </si>
+  <si>
+    <t>KMURRIETA</t>
+  </si>
+  <si>
+    <t>MAGNA ALOMIA CIELO</t>
+  </si>
+  <si>
+    <t>MAC</t>
+  </si>
+  <si>
+    <t>MONTECILLO DAVILA ROSITA TITIANA</t>
+  </si>
+  <si>
+    <t>MONROSITA</t>
+  </si>
+  <si>
+    <t>NUNEZ MERMAO VERONICA DEL PILAR</t>
+  </si>
+  <si>
+    <t>NUNEZVERO</t>
+  </si>
+  <si>
+    <t>NUÑEZ PACHECO, ENRIQUE</t>
+  </si>
+  <si>
+    <t>NPE</t>
+  </si>
+  <si>
+    <t>NUÑEZ PACHECO, PEDRO MIGUEL</t>
+  </si>
+  <si>
+    <t>NPPM</t>
+  </si>
+  <si>
+    <t>OFICINA</t>
+  </si>
+  <si>
+    <t>OF</t>
+  </si>
+  <si>
+    <t>PEGGY RENGIFO</t>
+  </si>
+  <si>
+    <t>PRENGIFO</t>
+  </si>
+  <si>
+    <t>RAMIREZ CARRASCO, KATTIA ANALY</t>
+  </si>
+  <si>
+    <t>RCKA</t>
+  </si>
+  <si>
+    <t>REBECA ELEONOR QUIROZ AMAYA</t>
+  </si>
+  <si>
+    <t>REQA</t>
+  </si>
+  <si>
+    <t>RETIZ CASTRO LISBETH</t>
+  </si>
+  <si>
+    <t>RETIZLISBETH</t>
+  </si>
+  <si>
+    <t>SAHARA ISABEL SAN BENTO AREVALO</t>
+  </si>
+  <si>
+    <t>SAS</t>
+  </si>
+  <si>
+    <t>SANDRA CAPILLO</t>
+  </si>
+  <si>
+    <t>THELMA MONICA PUJAY MARTINEZ</t>
+  </si>
+  <si>
+    <t>TMPM</t>
+  </si>
+  <si>
+    <t>VELA GALAN RUTH RAQUELI</t>
+  </si>
+  <si>
+    <t>VGRUTHR</t>
+  </si>
+  <si>
+    <t>YORK PAMELA</t>
+  </si>
+  <si>
+    <t>AUTOMOVIL</t>
+  </si>
+  <si>
+    <t>Activado</t>
+  </si>
+  <si>
+    <t>BARANDA</t>
+  </si>
+  <si>
+    <t>CAMION</t>
+  </si>
+  <si>
+    <t>CARRETA</t>
+  </si>
+  <si>
+    <t>CISTERNA</t>
+  </si>
+  <si>
+    <t>CMTA PANEL</t>
+  </si>
+  <si>
+    <t>CMTA PICK UP</t>
+  </si>
+  <si>
+    <t>CMTA RURAL MAYOR DE 9 ASIENTOS</t>
+  </si>
+  <si>
+    <t>FURGONETA</t>
+  </si>
+  <si>
+    <t>JIALING</t>
+  </si>
+  <si>
+    <t>MAQ. PESADA</t>
+  </si>
+  <si>
+    <t>MICROBUS</t>
+  </si>
+  <si>
+    <t>MINIBUS</t>
+  </si>
+  <si>
+    <t>MINIVAN</t>
+  </si>
+  <si>
+    <t>MOTOCICLETA</t>
+  </si>
+  <si>
+    <t>MOTOTAXI</t>
+  </si>
+  <si>
+    <t>OMNIBUS</t>
+  </si>
+  <si>
+    <t>REMOLCADOR</t>
+  </si>
+  <si>
+    <t>SEMI-REMOLQUE</t>
+  </si>
+  <si>
+    <t>VEHICULO MENOR</t>
+  </si>
+  <si>
+    <t>VOLQUETE&lt;12TON</t>
+  </si>
+  <si>
+    <t>VOLQUETE&gt;12TON</t>
+  </si>
+  <si>
+    <t>Costo Soat S/.   </t>
+  </si>
+  <si>
+    <t>Acción</t>
+  </si>
+  <si>
+    <t>ACTIVA</t>
+  </si>
+  <si>
+    <t>ADVANCE</t>
+  </si>
+  <si>
+    <t>ALESIN</t>
+  </si>
+  <si>
+    <t>ALEX</t>
+  </si>
+  <si>
+    <t>ALFA ROMEO</t>
+  </si>
+  <si>
+    <t>ALIMOTOR</t>
+  </si>
+  <si>
+    <t>AMAZON</t>
+  </si>
+  <si>
+    <t>ARLO</t>
+  </si>
+  <si>
+    <t>ARTSUN</t>
+  </si>
+  <si>
+    <t>ASIA HERO</t>
+  </si>
+  <si>
+    <t>AUDI</t>
+  </si>
+  <si>
+    <t>AZELLI</t>
+  </si>
+  <si>
+    <t>B52</t>
+  </si>
+  <si>
+    <t>BAIC</t>
+  </si>
+  <si>
+    <t>BAJAJ</t>
+  </si>
+  <si>
+    <t>BARSHA</t>
+  </si>
+  <si>
+    <t>BEAL</t>
+  </si>
+  <si>
+    <t>BENELLI</t>
+  </si>
+  <si>
+    <t>BJR</t>
+  </si>
+  <si>
+    <t>BMT</t>
+  </si>
+  <si>
+    <t>BMW</t>
+  </si>
+  <si>
+    <t>BOSUER</t>
+  </si>
+  <si>
+    <t>BRILLIANCE</t>
+  </si>
+  <si>
+    <t>BYD</t>
+  </si>
+  <si>
+    <t>C&amp;C MOTORS</t>
+  </si>
+  <si>
+    <t>CAMC</t>
+  </si>
+  <si>
+    <t>CAN-AM</t>
+  </si>
+  <si>
+    <t>CARGOMAX</t>
+  </si>
+  <si>
+    <t>CATERPILLAR</t>
+  </si>
+  <si>
+    <t>CF MOTO</t>
+  </si>
+  <si>
+    <t>CHANGAN</t>
+  </si>
+  <si>
+    <t>CHANGHE</t>
+  </si>
+  <si>
+    <t>CHERY</t>
+  </si>
+  <si>
+    <t>CHEVROLET</t>
+  </si>
+  <si>
+    <t>CHRYSLER</t>
+  </si>
+  <si>
+    <t>CITROEN</t>
+  </si>
+  <si>
+    <t>CMC</t>
+  </si>
+  <si>
+    <t>COBOS</t>
+  </si>
+  <si>
+    <t>COUNTY</t>
+  </si>
+  <si>
+    <t>CRICTOM</t>
+  </si>
+  <si>
+    <t>Email   </t>
+  </si>
+  <si>
+    <t>Teléfono   </t>
+  </si>
+  <si>
+    <t>Celular   </t>
+  </si>
+  <si>
+    <t>ALOMIA CIELO MAGNA</t>
+  </si>
+  <si>
+    <t>ALOMAGNA</t>
+  </si>
+  <si>
+    <t>ARIAS &amp; ARIAS CORREDORES DE SEGUROS SAC</t>
+  </si>
+  <si>
+    <t>AAS</t>
+  </si>
+  <si>
+    <t>ARIAS &amp; ARIAS CORREDORES DE SEGUROS SAC.</t>
+  </si>
+  <si>
+    <t>CESAR ARIAS</t>
+  </si>
+  <si>
+    <t>CAMARA DE COMERCIO INDUSTRIA Y TURISMO DE UCAYALI</t>
+  </si>
+  <si>
+    <t>CAM</t>
+  </si>
+  <si>
+    <t>cobranzas@camaraucayali.com</t>
+  </si>
+  <si>
+    <t>CAPILLO GABY</t>
+  </si>
+  <si>
+    <t>CASTILLOMARIAES</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTE Y SERVICIOS MULTIPLES ASMU SAC</t>
+  </si>
+  <si>
+    <t>ASM</t>
+  </si>
+  <si>
+    <t>Williams.calderon@hotmail.com</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTE Y SERVICIOS MULTIPLES EL SOL SAC.</t>
+  </si>
+  <si>
+    <t>ETYSMS</t>
+  </si>
+  <si>
+    <t>pedromiguelnupa2012@hotmail.com</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTE Y SERVICIOS MULTIPLES RAPS SAC</t>
+  </si>
+  <si>
+    <t>RAPS</t>
+  </si>
+  <si>
+    <t>Transportesraps2020@gmail.com</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTES &amp; SERVICIOS MULTIPLES TOURS CIELO AZUL SAC</t>
+  </si>
+  <si>
+    <t>CIE</t>
+  </si>
+  <si>
+    <t>TOURSCIELOAZUL@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTES Y MULTISERVCIOS GUESAN EIRL</t>
+  </si>
+  <si>
+    <t>GUES</t>
+  </si>
+  <si>
+    <t>guesan.eirl@gmail.com</t>
+  </si>
+  <si>
+    <t>EMPRESA DE TRANSPORTES Y SERVICIOS MULTIPLES AMOPROCOP SAC</t>
+  </si>
+  <si>
+    <t>AMO</t>
+  </si>
+  <si>
+    <t>Silviamoragrandez@gmail.com</t>
+  </si>
+  <si>
+    <t>FLORES HUAMANI ENRIQUE INOCENCIO</t>
+  </si>
+  <si>
+    <t>FLORESBE</t>
+  </si>
+  <si>
+    <t>Gabriela Ruiz Cespedes</t>
+  </si>
+  <si>
+    <t>985 040 531</t>
+  </si>
+  <si>
+    <t>KATTIA ANALY RAMIREZ CARRASCO</t>
+  </si>
+  <si>
+    <t>RCK</t>
+  </si>
+  <si>
+    <t>KATTY LOURDES BARDALES CAVIÑA</t>
+  </si>
+  <si>
+    <t>ESTRUCTURAS METÁLICA</t>
+  </si>
+  <si>
+    <t>INVERMARPUC@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>950 995 654</t>
+  </si>
+  <si>
+    <t>MONICA ANDION RUIZ</t>
+  </si>
+  <si>
+    <t>MONANRUIZ</t>
+  </si>
+  <si>
+    <t>chungandionnilo@gmail.com</t>
+  </si>
+  <si>
+    <t>MONICA ANDREA URIARTE ZAMORA</t>
+  </si>
+  <si>
+    <t>MAUZ</t>
+  </si>
+  <si>
+    <t>USUELROMA@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>961 621 800</t>
+  </si>
+  <si>
+    <t>QAR</t>
+  </si>
+  <si>
+    <t>REPRESENTACIONES VECTOR EIRL</t>
+  </si>
+  <si>
+    <t>VEC</t>
+  </si>
+  <si>
+    <t>fernando.vasuri@gmail.com</t>
+  </si>
+  <si>
+    <t>RIPPLE ORIENTE S.A.C</t>
+  </si>
+  <si>
+    <t>lauracanani@hotmail.com</t>
+  </si>
+  <si>
+    <t>943 036 797</t>
+  </si>
+  <si>
+    <t>945 175 818</t>
+  </si>
+  <si>
+    <t>SANDRA MILAGROS AVILA GOMEZ</t>
+  </si>
+  <si>
+    <t>COMERCIAL SANDRI</t>
+  </si>
+  <si>
+    <t>sandraavilagomez0308@gmail.com</t>
+  </si>
+  <si>
+    <t>TECNOLOGIA MOTRIZ EIRL</t>
+  </si>
+  <si>
+    <t>TECMO</t>
+  </si>
+  <si>
+    <t>administracion@gpstecnologiamotriz.com</t>
+  </si>
+  <si>
+    <t>MONPU</t>
+  </si>
+  <si>
+    <t>MONPUJ</t>
+  </si>
+  <si>
+    <t>TOYOMOTORS SRL</t>
+  </si>
+  <si>
+    <t>TOY</t>
+  </si>
+  <si>
+    <t>toyomotors3@hotmail.com</t>
+  </si>
+  <si>
+    <t>VGRUTH</t>
+  </si>
+  <si>
+    <t>VILLACORTA SORIA ANDREA</t>
+  </si>
+  <si>
+    <t>VILSANDREA</t>
+  </si>
+  <si>
+    <t>York Pamela Panduro Hidalgo</t>
+  </si>
+  <si>
+    <t>931 190 846</t>
+  </si>
+  <si>
+    <t>Name   </t>
+  </si>
+  <si>
+    <t>Privilege   </t>
+  </si>
+  <si>
+    <t>Photo   </t>
+  </si>
+  <si>
+    <t>Broke</t>
+  </si>
+  <si>
+    <t>JHORDIÑO RAMIREZ</t>
+  </si>
+  <si>
+    <t>tigestor@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>Broker</t>
+  </si>
+  <si>
+    <t>GIANELLY SABOYA</t>
+  </si>
+  <si>
+    <t>contabilidad@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>cesar-arias@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>DANIEL ARIAS</t>
+  </si>
+  <si>
+    <t>danielarias@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>KEVIN MURIETA</t>
+  </si>
+  <si>
+    <t>gestor@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>PAMELA PANDURO</t>
+  </si>
+  <si>
+    <t>soat@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>Operador</t>
+  </si>
+  <si>
+    <t>segurospersonales@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>coordinaciones@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>YURI GARCIA</t>
+  </si>
+  <si>
+    <t>yuri.garcia@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>peggy-rengifo@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>HUGO ARIAS</t>
+  </si>
+  <si>
+    <t>hugoarias@ways-solutions.com</t>
+  </si>
+  <si>
+    <t>BETTY FLORES</t>
+  </si>
+  <si>
+    <t>info@ariasyarias.com</t>
+  </si>
+  <si>
+    <t>  </t>
+  </si>
+  <si>
+    <t>URBANO/INTERURBANO</t>
+  </si>
+  <si>
+    <t>ESCOLAR</t>
+  </si>
+  <si>
+    <t>TRANSPORTE ESTUDIANTIL</t>
+  </si>
+  <si>
+    <t>TRANSPORTE PERSONAL</t>
+  </si>
+  <si>
+    <t>PUBLICO</t>
+  </si>
+  <si>
+    <t>RENTING</t>
+  </si>
+  <si>
+    <t>BOMBERO</t>
+  </si>
+  <si>
+    <t>AUTO COLECTIVO</t>
+  </si>
+  <si>
+    <t>A&amp;G AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd001</t>
+  </si>
+  <si>
+    <t>AAV AVIATION ADJUSTERS</t>
+  </si>
+  <si>
+    <t>AAV AVIATION</t>
+  </si>
+  <si>
+    <t>ajd002</t>
+  </si>
+  <si>
+    <t>ABACO PERU INTERNATIONAL LOSS ADJUSTERS AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ABACO PERU</t>
+  </si>
+  <si>
+    <t>ajd003</t>
+  </si>
+  <si>
+    <t>ACM AJUSTADORES Y PERITOS DE SEGUROS S.A.C</t>
+  </si>
+  <si>
+    <t>ACM AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd004</t>
+  </si>
+  <si>
+    <t>AFTER THE STORM</t>
+  </si>
+  <si>
+    <t>ajd005</t>
+  </si>
+  <si>
+    <t>APS AJUSTADORES Y PERITOS DE SEGUROS SRL</t>
+  </si>
+  <si>
+    <t>APS</t>
+  </si>
+  <si>
+    <t>ajd006</t>
+  </si>
+  <si>
+    <t>BAUKOST PERU</t>
+  </si>
+  <si>
+    <t>ajd007</t>
+  </si>
+  <si>
+    <t>Carlos Miguel Caro Custodio</t>
+  </si>
+  <si>
+    <t>Carlos Miguel Caro</t>
+  </si>
+  <si>
+    <t>ajd033</t>
+  </si>
+  <si>
+    <t>CESAR MONTOYA ALCANTARA</t>
+  </si>
+  <si>
+    <t>CESAR MONTOYA</t>
+  </si>
+  <si>
+    <t>ajd008</t>
+  </si>
+  <si>
+    <t>CHARLES TAYLOR AJUSTADORES DE SEGUROS S.A.</t>
+  </si>
+  <si>
+    <t>CHARLES TAYLOR</t>
+  </si>
+  <si>
+    <t>ajd009</t>
+  </si>
+  <si>
+    <t>COOPER BROTHERS</t>
+  </si>
+  <si>
+    <t>ajd010</t>
+  </si>
+  <si>
+    <t>CRAWFORD PERU S.A.</t>
+  </si>
+  <si>
+    <t>ajd011</t>
+  </si>
+  <si>
+    <t>GD AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd012</t>
+  </si>
+  <si>
+    <t>Gino Jesus Quispe Potesta</t>
+  </si>
+  <si>
+    <t>Gino Jesus Quispe</t>
+  </si>
+  <si>
+    <t>ajd034</t>
+  </si>
+  <si>
+    <t>HERRERA D.K.P.</t>
+  </si>
+  <si>
+    <t>ajd013</t>
+  </si>
+  <si>
+    <t>IRIARTE &amp; ASOCIADOS</t>
+  </si>
+  <si>
+    <t>IRIARTE</t>
+  </si>
+  <si>
+    <t>ajd014</t>
+  </si>
+  <si>
+    <t>J.R.Z. AJUSTADORES Y PERITOS DE SEGUROS</t>
+  </si>
+  <si>
+    <t>J.R.Z. AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd015</t>
+  </si>
+  <si>
+    <t>JORGE VALVERDE</t>
+  </si>
+  <si>
+    <t>ajd016</t>
+  </si>
+  <si>
+    <t>LA BRITANICA</t>
+  </si>
+  <si>
+    <t>ajd017</t>
+  </si>
+  <si>
+    <t>MARIO EDY GUILLERMO ARRATEA QUISPE</t>
+  </si>
+  <si>
+    <t>MARIO EDY GUILLERMO</t>
+  </si>
+  <si>
+    <t>ajd032</t>
+  </si>
+  <si>
+    <t>MASTER AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd018</t>
+  </si>
+  <si>
+    <t>MIGUEL ANGEL NUNEZ SANCHEZ</t>
+  </si>
+  <si>
+    <t>MIGUEL ANGEL NUNEZ</t>
+  </si>
+  <si>
+    <t>ajd036</t>
+  </si>
+  <si>
+    <t>OSBERK</t>
+  </si>
+  <si>
+    <t>ajd019</t>
+  </si>
+  <si>
+    <t>PABLO VIGO</t>
+  </si>
+  <si>
+    <t>ajd020</t>
+  </si>
+  <si>
+    <t>PERU VERITAS</t>
+  </si>
+  <si>
+    <t>ajd021</t>
+  </si>
+  <si>
+    <t>PREVENCION Y CONTROL</t>
+  </si>
+  <si>
+    <t>ajd022</t>
+  </si>
+  <si>
+    <t>Protegia Ajustadores</t>
+  </si>
+  <si>
+    <t>ADJ037</t>
+  </si>
+  <si>
+    <t>RAUL ARBOCCO LICETI</t>
+  </si>
+  <si>
+    <t>ajd024</t>
+  </si>
+  <si>
+    <t>ROMERO AJUSTADORES SRL</t>
+  </si>
+  <si>
+    <t>ROMERO AJUSTADORES</t>
+  </si>
+  <si>
+    <t>ajd023</t>
+  </si>
+  <si>
+    <t>RTS-PERU PERITOS Y AJUSTADORES DE SEGUROS S.A.C.</t>
+  </si>
+  <si>
+    <t>RTS-PERU</t>
+  </si>
+  <si>
+    <t>ajd025</t>
+  </si>
+  <si>
+    <t>S.O.S SEGURIDAD OPERACIONES  SALVATAJE</t>
+  </si>
+  <si>
+    <t>S.O.S SEGURIDAD</t>
+  </si>
+  <si>
+    <t>ajd026</t>
+  </si>
+  <si>
+    <t>Saenz &amp; Asociados Ajustadores de Seguros SAC</t>
+  </si>
+  <si>
+    <t>Saenz &amp; Asociados</t>
+  </si>
+  <si>
+    <t>ajd035</t>
+  </si>
+  <si>
+    <t>SUPERVISIONES &amp; PREVENCIONES S.R.L. AJUSTADORES Y PERITOS DE SEGUROS</t>
+  </si>
+  <si>
+    <t>SUPERV &amp; PREVEN</t>
+  </si>
+  <si>
+    <t>ajd027</t>
+  </si>
+  <si>
+    <t>TEODORO MONTENEGRO</t>
+  </si>
+  <si>
+    <t>ajd028</t>
+  </si>
+  <si>
+    <t>TRANSATLANTIC</t>
+  </si>
+  <si>
+    <t>ajd029</t>
+  </si>
+  <si>
+    <t>VILLNUEVE NAVAL ENGINEERS SRL</t>
+  </si>
+  <si>
+    <t>VILLNUEVE NAVAL</t>
+  </si>
+  <si>
+    <t>ajd030</t>
+  </si>
+  <si>
+    <t>W.MOLLER</t>
+  </si>
+  <si>
+    <t>ajd031</t>
+  </si>
+  <si>
+    <t>BANCO BBVA PERU</t>
+  </si>
+  <si>
+    <t>BANCO DE CREDITO DEL PERU</t>
+  </si>
+  <si>
+    <t>BANCO INTERAMERICANO DE FINANZAS</t>
+  </si>
+  <si>
+    <t>BANCO INTERBANK</t>
+  </si>
+  <si>
+    <t>BANCO SANTANDER PERU S.A</t>
+  </si>
+  <si>
+    <t>BBVA + BCP</t>
+  </si>
+  <si>
+    <t>BBVA CONSUMER FINANCE - EDPYME</t>
+  </si>
+  <si>
+    <t>BCP+BBVA+INTERBANK+SCOTIABANK</t>
+  </si>
+  <si>
+    <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE MAYNAS S.A.</t>
+  </si>
+  <si>
+    <t>CATERPILLAR LEASING CHILE S.A</t>
+  </si>
+  <si>
+    <t>CGM RENTAL SAC</t>
+  </si>
+  <si>
+    <t>CMAC PIURA SAC</t>
+  </si>
+  <si>
+    <t>EDPYME SANTANDER CONSUMO PERU SA</t>
+  </si>
+  <si>
+    <t>EMPRESA DE CREDITOS SANTANDER CONSUMO PERU S.A.</t>
+  </si>
+  <si>
+    <t>FORUM DISTRIBUIDORA DEL PERU S.A.</t>
+  </si>
+  <si>
+    <t>ITRALTAC SELVA SAC</t>
+  </si>
+  <si>
+    <t>JOHN DEERE FINANCIAL CHILE SPA</t>
+  </si>
+  <si>
+    <t>KOMATSU-MITSUI MAQUINARIAS PERU S.A.</t>
+  </si>
+  <si>
+    <t>MARANON HEAVY EQUIPMENT SAC</t>
+  </si>
+  <si>
+    <t>MITSUI AUTO FINANCE PERU SA</t>
+  </si>
+  <si>
+    <t>ORVISA SA</t>
+  </si>
+  <si>
+    <t>PAGO EFECTIVO</t>
+  </si>
+  <si>
+    <t>PANDERO S.A. EAFC</t>
+  </si>
+  <si>
+    <t>PROMOTORA OPCION S.A. EAFC</t>
+  </si>
+  <si>
+    <t>SCOTIABANK PERU SAA</t>
+  </si>
+  <si>
+    <t>ZOOMLION HEAVY INDUSTRY PERU S.A.C.</t>
+  </si>
+  <si>
+    <t>Marcas Id   </t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>116I</t>
+  </si>
+  <si>
+    <t>523I</t>
+  </si>
+  <si>
+    <t>318I</t>
+  </si>
+  <si>
+    <t>640I</t>
+  </si>
+  <si>
+    <t>330CI</t>
+  </si>
+  <si>
+    <t>X6</t>
+  </si>
+  <si>
+    <t>118i</t>
+  </si>
+  <si>
+    <t>525I</t>
+  </si>
+  <si>
+    <t>318is</t>
+  </si>
+  <si>
+    <t>730I</t>
+  </si>
+  <si>
+    <t>330d</t>
+  </si>
+  <si>
+    <t>120I</t>
+  </si>
+  <si>
+    <t>528I</t>
+  </si>
+  <si>
+    <t>320CI</t>
+  </si>
+  <si>
+    <t>735I</t>
+  </si>
+  <si>
+    <t>330I</t>
+  </si>
+  <si>
+    <t>125I</t>
+  </si>
+  <si>
+    <t>530D</t>
+  </si>
+  <si>
+    <t>320D</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +2234,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1057,8 +2270,37 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1089,6 +2331,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1099,11 +2353,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1111,12 +2366,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -11768,4 +13091,2905 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{052E6A8E-6303-4CFC-85C2-38CC10A11689}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C2" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>568</v>
+      </c>
+      <c r="B3" t="s">
+        <v>404</v>
+      </c>
+      <c r="C3" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B4" t="s">
+        <v>404</v>
+      </c>
+      <c r="C4" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>569</v>
+      </c>
+      <c r="B6" t="s">
+        <v>404</v>
+      </c>
+      <c r="C6" t="s">
+        <v>567</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>570</v>
+      </c>
+      <c r="B7" t="s">
+        <v>404</v>
+      </c>
+      <c r="C7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>571</v>
+      </c>
+      <c r="B8" t="s">
+        <v>404</v>
+      </c>
+      <c r="C8" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" t="s">
+        <v>404</v>
+      </c>
+      <c r="C9" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" t="s">
+        <v>404</v>
+      </c>
+      <c r="C10" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>572</v>
+      </c>
+      <c r="B11" t="s">
+        <v>404</v>
+      </c>
+      <c r="C11" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>573</v>
+      </c>
+      <c r="B12" t="s">
+        <v>404</v>
+      </c>
+      <c r="C12" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" t="s">
+        <v>404</v>
+      </c>
+      <c r="C13" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>574</v>
+      </c>
+      <c r="B14" t="s">
+        <v>404</v>
+      </c>
+      <c r="C14" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>575</v>
+      </c>
+      <c r="B15" t="s">
+        <v>404</v>
+      </c>
+      <c r="C15" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B16" t="s">
+        <v>404</v>
+      </c>
+      <c r="C16" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" t="s">
+        <v>404</v>
+      </c>
+      <c r="C17" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" t="s">
+        <v>404</v>
+      </c>
+      <c r="C18" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" t="s">
+        <v>404</v>
+      </c>
+      <c r="C19" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>187</v>
+      </c>
+      <c r="B20" t="s">
+        <v>404</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A20">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{005A5A4A-BD6C-4E3B-9C34-6F72B7AB1BEE}">
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>576</v>
+      </c>
+      <c r="B2" t="s">
+        <v>576</v>
+      </c>
+      <c r="C2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>578</v>
+      </c>
+      <c r="B3" t="s">
+        <v>579</v>
+      </c>
+      <c r="C3" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>581</v>
+      </c>
+      <c r="B4" t="s">
+        <v>582</v>
+      </c>
+      <c r="C4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>584</v>
+      </c>
+      <c r="B5" t="s">
+        <v>585</v>
+      </c>
+      <c r="C5" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>587</v>
+      </c>
+      <c r="B6" t="s">
+        <v>587</v>
+      </c>
+      <c r="C6" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>589</v>
+      </c>
+      <c r="B7" t="s">
+        <v>590</v>
+      </c>
+      <c r="C7" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>592</v>
+      </c>
+      <c r="B8" t="s">
+        <v>592</v>
+      </c>
+      <c r="C8" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>594</v>
+      </c>
+      <c r="B9" t="s">
+        <v>595</v>
+      </c>
+      <c r="C9" t="s">
+        <v>596</v>
+      </c>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>597</v>
+      </c>
+      <c r="B10" t="s">
+        <v>598</v>
+      </c>
+      <c r="C10" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>600</v>
+      </c>
+      <c r="B11" t="s">
+        <v>601</v>
+      </c>
+      <c r="C11" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>603</v>
+      </c>
+      <c r="B12" t="s">
+        <v>603</v>
+      </c>
+      <c r="C12" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>605</v>
+      </c>
+      <c r="B13" t="s">
+        <v>605</v>
+      </c>
+      <c r="C13" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>607</v>
+      </c>
+      <c r="B14" t="s">
+        <v>607</v>
+      </c>
+      <c r="C14" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>609</v>
+      </c>
+      <c r="B15" t="s">
+        <v>610</v>
+      </c>
+      <c r="C15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>612</v>
+      </c>
+      <c r="B16" t="s">
+        <v>612</v>
+      </c>
+      <c r="C16" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>614</v>
+      </c>
+      <c r="B17" t="s">
+        <v>615</v>
+      </c>
+      <c r="C17" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>617</v>
+      </c>
+      <c r="B18" t="s">
+        <v>618</v>
+      </c>
+      <c r="C18" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>620</v>
+      </c>
+      <c r="B19" t="s">
+        <v>620</v>
+      </c>
+      <c r="C19" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>622</v>
+      </c>
+      <c r="B20" t="s">
+        <v>622</v>
+      </c>
+      <c r="C20" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>624</v>
+      </c>
+      <c r="B21" t="s">
+        <v>625</v>
+      </c>
+      <c r="C21" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>627</v>
+      </c>
+      <c r="B22" t="s">
+        <v>627</v>
+      </c>
+      <c r="C22" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>629</v>
+      </c>
+      <c r="B23" t="s">
+        <v>630</v>
+      </c>
+      <c r="C23" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>632</v>
+      </c>
+      <c r="B24" t="s">
+        <v>632</v>
+      </c>
+      <c r="C24" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>634</v>
+      </c>
+      <c r="B25" t="s">
+        <v>634</v>
+      </c>
+      <c r="C25" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>636</v>
+      </c>
+      <c r="B26" t="s">
+        <v>636</v>
+      </c>
+      <c r="C26" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>638</v>
+      </c>
+      <c r="B27" t="s">
+        <v>638</v>
+      </c>
+      <c r="C27" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>640</v>
+      </c>
+      <c r="B28" t="s">
+        <v>640</v>
+      </c>
+      <c r="C28" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>642</v>
+      </c>
+      <c r="B29" t="s">
+        <v>642</v>
+      </c>
+      <c r="C29" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>644</v>
+      </c>
+      <c r="B30" t="s">
+        <v>645</v>
+      </c>
+      <c r="C30" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>647</v>
+      </c>
+      <c r="B31" t="s">
+        <v>648</v>
+      </c>
+      <c r="C31" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>650</v>
+      </c>
+      <c r="B32" t="s">
+        <v>651</v>
+      </c>
+      <c r="C32" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>653</v>
+      </c>
+      <c r="B33" t="s">
+        <v>654</v>
+      </c>
+      <c r="C33" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>656</v>
+      </c>
+      <c r="B34" t="s">
+        <v>657</v>
+      </c>
+      <c r="C34" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>659</v>
+      </c>
+      <c r="B35" t="s">
+        <v>659</v>
+      </c>
+      <c r="C35" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>661</v>
+      </c>
+      <c r="B36" t="s">
+        <v>661</v>
+      </c>
+      <c r="C36" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>663</v>
+      </c>
+      <c r="B37" t="s">
+        <v>664</v>
+      </c>
+      <c r="C37" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>666</v>
+      </c>
+      <c r="B38" t="s">
+        <v>666</v>
+      </c>
+      <c r="C38" t="s">
+        <v>667</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A38">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32C25434-05B0-49D5-8DA8-46861818293E}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="21.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2">
+        <v>10098695899</v>
+      </c>
+      <c r="D2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="B3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C3">
+        <v>10098695898</v>
+      </c>
+      <c r="E3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>325</v>
+      </c>
+      <c r="B5" t="s">
+        <v>325</v>
+      </c>
+      <c r="E5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B6" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B7" t="s">
+        <v>330</v>
+      </c>
+      <c r="C7">
+        <v>20523470761</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B8" t="s">
+        <v>332</v>
+      </c>
+      <c r="C8">
+        <v>20600098633</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>333</v>
+      </c>
+      <c r="B9" t="s">
+        <v>334</v>
+      </c>
+      <c r="C9">
+        <v>20454073143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="B10" t="s">
+        <v>336</v>
+      </c>
+      <c r="C10">
+        <v>20601978572</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="B11" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11">
+        <v>20517207331</v>
+      </c>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>339</v>
+      </c>
+      <c r="B12" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>340</v>
+      </c>
+      <c r="B13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C13">
+        <v>20553157014</v>
+      </c>
+      <c r="D13" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>343</v>
+      </c>
+      <c r="B14" t="s">
+        <v>344</v>
+      </c>
+      <c r="C14">
+        <v>20554816526</v>
+      </c>
+      <c r="D14" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>346</v>
+      </c>
+      <c r="B15" t="s">
+        <v>347</v>
+      </c>
+      <c r="C15">
+        <v>20610079777</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{220DC1E9-AAD2-4C53-AA9A-04F42D4CE81E}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>355</v>
+      </c>
+      <c r="B6" t="s">
+        <v>356</v>
+      </c>
+      <c r="C6" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>357</v>
+      </c>
+      <c r="B7" t="s">
+        <v>358</v>
+      </c>
+      <c r="C7" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B8" t="s">
+        <v>360</v>
+      </c>
+      <c r="C8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>361</v>
+      </c>
+      <c r="B9" t="s">
+        <v>362</v>
+      </c>
+      <c r="C9" t="s">
+        <v>307</v>
+      </c>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>363</v>
+      </c>
+      <c r="B10" t="s">
+        <v>364</v>
+      </c>
+      <c r="C10" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>365</v>
+      </c>
+      <c r="B11" t="s">
+        <v>366</v>
+      </c>
+      <c r="C11" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>369</v>
+      </c>
+      <c r="B13" t="s">
+        <v>370</v>
+      </c>
+      <c r="C13" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>371</v>
+      </c>
+      <c r="B14" t="s">
+        <v>372</v>
+      </c>
+      <c r="C14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>375</v>
+      </c>
+      <c r="B16" t="s">
+        <v>376</v>
+      </c>
+      <c r="C16" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>377</v>
+      </c>
+      <c r="B17" t="s">
+        <v>378</v>
+      </c>
+      <c r="C17" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>379</v>
+      </c>
+      <c r="B18" t="s">
+        <v>380</v>
+      </c>
+      <c r="C18" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>389</v>
+      </c>
+      <c r="B23" t="s">
+        <v>390</v>
+      </c>
+      <c r="C23" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>391</v>
+      </c>
+      <c r="B24" t="s">
+        <v>392</v>
+      </c>
+      <c r="C24" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>393</v>
+      </c>
+      <c r="B25" t="s">
+        <v>394</v>
+      </c>
+      <c r="C25" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>395</v>
+      </c>
+      <c r="B26" t="s">
+        <v>396</v>
+      </c>
+      <c r="C26" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>398</v>
+      </c>
+      <c r="B28" t="s">
+        <v>399</v>
+      </c>
+      <c r="C28" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>400</v>
+      </c>
+      <c r="B29" t="s">
+        <v>401</v>
+      </c>
+      <c r="C29" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{354DA039-CB2D-446D-9C95-9A79489222F4}">
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="49.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>668</v>
+      </c>
+      <c r="B2" s="12"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>669</v>
+      </c>
+      <c r="B3" s="12"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>670</v>
+      </c>
+      <c r="B4" s="12"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>671</v>
+      </c>
+      <c r="B5" s="12"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>672</v>
+      </c>
+      <c r="B6" s="12"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>673</v>
+      </c>
+      <c r="B7" s="12"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>674</v>
+      </c>
+      <c r="B8" s="12"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>675</v>
+      </c>
+      <c r="B9" s="12"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>676</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>677</v>
+      </c>
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>678</v>
+      </c>
+      <c r="B12" s="12"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>679</v>
+      </c>
+      <c r="B13" s="12"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>680</v>
+      </c>
+      <c r="B14" s="12"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>681</v>
+      </c>
+      <c r="B15" s="12"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>682</v>
+      </c>
+      <c r="B16" s="12"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>683</v>
+      </c>
+      <c r="B17" s="12"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>684</v>
+      </c>
+      <c r="B18" s="12"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>685</v>
+      </c>
+      <c r="B19" s="12"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>686</v>
+      </c>
+      <c r="B20" s="12"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>687</v>
+      </c>
+      <c r="B21" s="12"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>688</v>
+      </c>
+      <c r="B22" s="12"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>689</v>
+      </c>
+      <c r="B23" s="12"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>690</v>
+      </c>
+      <c r="B24" s="12"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>691</v>
+      </c>
+      <c r="B25" s="12"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>692</v>
+      </c>
+      <c r="B26" s="12"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>693</v>
+      </c>
+      <c r="B27" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78F2D09D-7DDD-4CDD-986F-F5A08AE1205D}">
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>405</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>407</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>408</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>410</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>412</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
+        <v>404</v>
+      </c>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>414</v>
+      </c>
+      <c r="B12">
+        <v>270</v>
+      </c>
+      <c r="C12" t="s">
+        <v>404</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>415</v>
+      </c>
+      <c r="B13" s="8">
+        <v>0</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>416</v>
+      </c>
+      <c r="B14">
+        <v>630</v>
+      </c>
+      <c r="C14" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="B15" s="8">
+        <v>0</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>418</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>419</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>420</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>421</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>422</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>423</v>
+      </c>
+      <c r="B21">
+        <v>50</v>
+      </c>
+      <c r="C21" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>424</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>425</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F24" s="7"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A23">
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F52191DD-DE2E-41AC-B908-70F1ABE6C0CC}">
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>430</v>
+      </c>
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>431</v>
+      </c>
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>432</v>
+      </c>
+      <c r="C6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>433</v>
+      </c>
+      <c r="C7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>434</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>435</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>436</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>437</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>438</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>439</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>440</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>441</v>
+      </c>
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>442</v>
+      </c>
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>443</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>444</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>445</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>446</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>448</v>
+      </c>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>449</v>
+      </c>
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>450</v>
+      </c>
+      <c r="C24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>451</v>
+      </c>
+      <c r="C25" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>452</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>453</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>454</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>455</v>
+      </c>
+      <c r="C29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>456</v>
+      </c>
+      <c r="C30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>457</v>
+      </c>
+      <c r="C31" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>458</v>
+      </c>
+      <c r="C32" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>459</v>
+      </c>
+      <c r="C33" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>460</v>
+      </c>
+      <c r="C34" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>461</v>
+      </c>
+      <c r="C35" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>462</v>
+      </c>
+      <c r="C36" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>463</v>
+      </c>
+      <c r="C37" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>464</v>
+      </c>
+      <c r="C38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>465</v>
+      </c>
+      <c r="C39" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>466</v>
+      </c>
+      <c r="C40" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>467</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E14834B2-4090-49F7-A48A-10F36CAA051F}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B2" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>448</v>
+      </c>
+      <c r="B3" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>448</v>
+      </c>
+      <c r="B4" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>448</v>
+      </c>
+      <c r="B5" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>448</v>
+      </c>
+      <c r="B6" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>448</v>
+      </c>
+      <c r="B7" t="s">
+        <v>700</v>
+      </c>
+      <c r="D7" t="s">
+        <v>567</v>
+      </c>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>448</v>
+      </c>
+      <c r="B8" t="s">
+        <v>701</v>
+      </c>
+      <c r="D8" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>448</v>
+      </c>
+      <c r="B9" t="s">
+        <v>702</v>
+      </c>
+      <c r="D9" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>448</v>
+      </c>
+      <c r="B10" t="s">
+        <v>703</v>
+      </c>
+      <c r="D10" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>448</v>
+      </c>
+      <c r="B11" t="s">
+        <v>704</v>
+      </c>
+      <c r="D11" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>448</v>
+      </c>
+      <c r="B12" t="s">
+        <v>705</v>
+      </c>
+      <c r="D12" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>448</v>
+      </c>
+      <c r="B13" t="s">
+        <v>706</v>
+      </c>
+      <c r="D13" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>448</v>
+      </c>
+      <c r="B14" t="s">
+        <v>707</v>
+      </c>
+      <c r="D14" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>448</v>
+      </c>
+      <c r="B15" t="s">
+        <v>708</v>
+      </c>
+      <c r="D15" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>448</v>
+      </c>
+      <c r="B16" t="s">
+        <v>709</v>
+      </c>
+      <c r="D16" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>448</v>
+      </c>
+      <c r="B17" t="s">
+        <v>710</v>
+      </c>
+      <c r="D17" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>448</v>
+      </c>
+      <c r="B18" t="s">
+        <v>711</v>
+      </c>
+      <c r="D18" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>448</v>
+      </c>
+      <c r="B19" t="s">
+        <v>712</v>
+      </c>
+      <c r="D19" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>448</v>
+      </c>
+      <c r="B20" t="s">
+        <v>713</v>
+      </c>
+      <c r="D20" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>448</v>
+      </c>
+      <c r="B21" t="s">
+        <v>714</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8CC615C-A336-47F2-ADD8-55FAA0EF421E}">
+  <dimension ref="A1:F42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B2" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>473</v>
+      </c>
+      <c r="B3" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>475</v>
+      </c>
+      <c r="B4" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="B5" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>355</v>
+      </c>
+      <c r="B6" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>477</v>
+      </c>
+      <c r="B7" t="s">
+        <v>478</v>
+      </c>
+      <c r="C7" t="s">
+        <v>479</v>
+      </c>
+      <c r="D7">
+        <v>986670400</v>
+      </c>
+      <c r="E7">
+        <v>986670400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B8" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>361</v>
+      </c>
+      <c r="B9" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>482</v>
+      </c>
+      <c r="B10" t="s">
+        <v>483</v>
+      </c>
+      <c r="C10" t="s">
+        <v>484</v>
+      </c>
+      <c r="D10">
+        <v>983910086</v>
+      </c>
+      <c r="E10">
+        <v>983910086</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>485</v>
+      </c>
+      <c r="B11" t="s">
+        <v>486</v>
+      </c>
+      <c r="C11" t="s">
+        <v>487</v>
+      </c>
+      <c r="E11">
+        <v>965880494</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>488</v>
+      </c>
+      <c r="B12" t="s">
+        <v>489</v>
+      </c>
+      <c r="C12" t="s">
+        <v>490</v>
+      </c>
+      <c r="D12">
+        <v>932736846</v>
+      </c>
+      <c r="E12">
+        <v>932736846</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>491</v>
+      </c>
+      <c r="B13" t="s">
+        <v>492</v>
+      </c>
+      <c r="C13" t="s">
+        <v>493</v>
+      </c>
+      <c r="D13">
+        <v>971248974</v>
+      </c>
+      <c r="E13">
+        <v>971248974</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>494</v>
+      </c>
+      <c r="B14" t="s">
+        <v>495</v>
+      </c>
+      <c r="C14" t="s">
+        <v>496</v>
+      </c>
+      <c r="D14">
+        <v>910820923</v>
+      </c>
+      <c r="E14">
+        <v>910820923</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>497</v>
+      </c>
+      <c r="B15" t="s">
+        <v>498</v>
+      </c>
+      <c r="C15" t="s">
+        <v>499</v>
+      </c>
+      <c r="D15">
+        <v>913049639</v>
+      </c>
+      <c r="E15">
+        <v>913049639</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>500</v>
+      </c>
+      <c r="B16" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
+        <v>502</v>
+      </c>
+      <c r="B17" t="s">
+        <v>367</v>
+      </c>
+      <c r="E17" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>504</v>
+      </c>
+      <c r="B18" t="s">
+        <v>505</v>
+      </c>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>506</v>
+      </c>
+      <c r="B19" t="s">
+        <v>507</v>
+      </c>
+      <c r="C19" t="s">
+        <v>508</v>
+      </c>
+      <c r="D19">
+        <v>982501583</v>
+      </c>
+      <c r="E19">
+        <v>982501583</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="B20" t="s">
+        <v>373</v>
+      </c>
+      <c r="E20" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>510</v>
+      </c>
+      <c r="B21" t="s">
+        <v>511</v>
+      </c>
+      <c r="C21" t="s">
+        <v>512</v>
+      </c>
+      <c r="D21">
+        <v>966220272</v>
+      </c>
+      <c r="E21">
+        <v>966220272</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>513</v>
+      </c>
+      <c r="B22" t="s">
+        <v>514</v>
+      </c>
+      <c r="C22" t="s">
+        <v>515</v>
+      </c>
+      <c r="D22">
+        <v>949452389</v>
+      </c>
+      <c r="E22">
+        <v>949452389</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="B23" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>391</v>
+      </c>
+      <c r="B24" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>518</v>
+      </c>
+      <c r="B25" t="s">
+        <v>519</v>
+      </c>
+      <c r="C25" t="s">
+        <v>520</v>
+      </c>
+      <c r="D25">
+        <v>983601295</v>
+      </c>
+      <c r="E25">
+        <v>983601295</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>393</v>
+      </c>
+      <c r="B26" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>521</v>
+      </c>
+      <c r="B27" t="s">
+        <v>521</v>
+      </c>
+      <c r="C27" t="s">
+        <v>522</v>
+      </c>
+      <c r="E27" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>395</v>
+      </c>
+      <c r="B28" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>395</v>
+      </c>
+      <c r="B29" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>395</v>
+      </c>
+      <c r="B30" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>395</v>
+      </c>
+      <c r="B31" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="B32" t="s">
+        <v>397</v>
+      </c>
+      <c r="E32" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>525</v>
+      </c>
+      <c r="B33" t="s">
+        <v>526</v>
+      </c>
+      <c r="C33" t="s">
+        <v>527</v>
+      </c>
+      <c r="E33">
+        <v>961776502</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>528</v>
+      </c>
+      <c r="B34" t="s">
+        <v>529</v>
+      </c>
+      <c r="C34" t="s">
+        <v>530</v>
+      </c>
+      <c r="D34">
+        <v>933600666</v>
+      </c>
+      <c r="E34">
+        <v>933600666</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>398</v>
+      </c>
+      <c r="B35" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>398</v>
+      </c>
+      <c r="B36" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>398</v>
+      </c>
+      <c r="B37" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>533</v>
+      </c>
+      <c r="B38" t="s">
+        <v>534</v>
+      </c>
+      <c r="C38" t="s">
+        <v>535</v>
+      </c>
+      <c r="D38">
+        <v>961501225</v>
+      </c>
+      <c r="E38">
+        <v>961501225</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>400</v>
+      </c>
+      <c r="B39" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>400</v>
+      </c>
+      <c r="B40" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>537</v>
+      </c>
+      <c r="B41" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="10" t="s">
+        <v>539</v>
+      </c>
+      <c r="B42" t="s">
+        <v>402</v>
+      </c>
+      <c r="E42" t="s">
+        <v>540</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A42">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5421208-44B4-409F-8F02-C8815EC1BD9E}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C2" t="s">
+        <v>547</v>
+      </c>
+      <c r="E2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>548</v>
+      </c>
+      <c r="B3" t="s">
+        <v>549</v>
+      </c>
+      <c r="C3" t="s">
+        <v>547</v>
+      </c>
+      <c r="E3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>476</v>
+      </c>
+      <c r="B4" t="s">
+        <v>550</v>
+      </c>
+      <c r="C4" t="s">
+        <v>547</v>
+      </c>
+      <c r="E4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>551</v>
+      </c>
+      <c r="B5" t="s">
+        <v>552</v>
+      </c>
+      <c r="C5" t="s">
+        <v>547</v>
+      </c>
+      <c r="E5" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>553</v>
+      </c>
+      <c r="B6" t="s">
+        <v>554</v>
+      </c>
+      <c r="C6" t="s">
+        <v>547</v>
+      </c>
+      <c r="E6" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>555</v>
+      </c>
+      <c r="B7" t="s">
+        <v>556</v>
+      </c>
+      <c r="C7" t="s">
+        <v>557</v>
+      </c>
+      <c r="E7" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>397</v>
+      </c>
+      <c r="B8" t="s">
+        <v>558</v>
+      </c>
+      <c r="C8" t="s">
+        <v>557</v>
+      </c>
+      <c r="E8" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>367</v>
+      </c>
+      <c r="B9" t="s">
+        <v>559</v>
+      </c>
+      <c r="C9" t="s">
+        <v>557</v>
+      </c>
+      <c r="E9" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>560</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="C10" t="s">
+        <v>547</v>
+      </c>
+      <c r="E10" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>387</v>
+      </c>
+      <c r="B11" t="s">
+        <v>562</v>
+      </c>
+      <c r="C11" t="s">
+        <v>547</v>
+      </c>
+      <c r="E11" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>563</v>
+      </c>
+      <c r="B12" t="s">
+        <v>564</v>
+      </c>
+      <c r="C12" t="s">
+        <v>547</v>
+      </c>
+      <c r="E12" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>565</v>
+      </c>
+      <c r="B13" t="s">
+        <v>566</v>
+      </c>
+      <c r="C13" t="s">
+        <v>547</v>
+      </c>
+      <c r="E13" t="s">
+        <v>475</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{CF70C26B-8537-4B26-9478-F07CF0CAC2AA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>